<commit_message>
Dodano youtube opcija i sitne dorde u dizajnu
</commit_message>
<xml_diff>
--- a/bandhelper_final_ui_ready_v5.xlsx
+++ b/bandhelper_final_ui_ready_v5.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11010"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10912"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mara/Apps/Repertoar_app/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/markomarjanovic/Apps/Repertoar_app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D82AF011-A459-674F-A3E1-448A802EFF9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{524D724C-D995-2345-B299-38336DD02396}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="460" windowWidth="38160" windowHeight="21140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,19 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="50">
-  <si>
-    <t>title</t>
-  </si>
-  <si>
-    <t>artist</t>
-  </si>
-  <si>
-    <t>key</t>
-  </si>
-  <si>
-    <t>tempo</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="68">
   <si>
     <t>region</t>
   </si>
@@ -46,9 +34,6 @@
     <t>lyrics</t>
   </si>
   <si>
-    <t>origin</t>
-  </si>
-  <si>
     <t>theme</t>
   </si>
   <si>
@@ -56,12 +41,6 @@
   </si>
   <si>
     <t>Srednja</t>
-  </si>
-  <si>
-    <t>genre</t>
-  </si>
-  <si>
-    <t>instrumental</t>
   </si>
   <si>
     <t>Opet je jubin cilin tilom</t>
@@ -480,6 +459,169 @@
   </si>
   <si>
     <t>BIH</t>
+  </si>
+  <si>
+    <t>title*</t>
+  </si>
+  <si>
+    <t>artist*</t>
+  </si>
+  <si>
+    <t>key*</t>
+  </si>
+  <si>
+    <t>tempo*</t>
+  </si>
+  <si>
+    <t>genre*</t>
+  </si>
+  <si>
+    <t>origin*</t>
+  </si>
+  <si>
+    <t>vocal*</t>
+  </si>
+  <si>
+    <t>Muško</t>
+  </si>
+  <si>
+    <t>Žensko</t>
+  </si>
+  <si>
+    <t>is_instrumental</t>
+  </si>
+  <si>
+    <t>score_pdf</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>Ja pijem da zaboravim</t>
+  </si>
+  <si>
+    <t>Moj je Dado puno radio</t>
+  </si>
+  <si>
+    <t>Gazde</t>
+  </si>
+  <si>
+    <t>Tambure</t>
+  </si>
+  <si>
+    <t>TS Zvona</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>Slavonija</t>
+  </si>
+  <si>
+    <t>Moj je dado puno radio
+a ja samo novce trosio
+ja k'o gazda, on k'o sluga
+sad imamo zbog tog duga
+moj je dado puno radio
+Kada zorom sunce osvane
+mene svirci kuci doprate
+pet sviraca mene prati
+'ajde, dado, ti im plati
+nis' me valjda dzabe pratili
+Kaze dado - 'ajmo raditi
+valjalo bi zito kositi
+pusti, dado, zito, sijeno
+bas je vruce, cudo jedno
+'ajmo, dado, stogod popiti
+Dok je meni dade u kuci
+u zivotu nis' me ne muci
+dado radi, meni daje
+sto je lipo neka traje
+da se dadi sto god ne desi</t>
+  </si>
+  <si>
+    <t>Od tebe sam, mala, bjezao
+bez tebe sam budan lezao
+zbog tebe sam sto zivota tudjih slomio
+al' od sebe nisam pobjeg'o
+Tvoje srce cisto, nevino
+priznajem da nisam shvatio
+ja sam htio puno vise, ruzu ubrati
+ti me nisi mogla pratiti
+Ref. 2x
+Ja pijem da zaboravim
+ja kockam da se umorim
+moj je broj odavno pao
+kad sam tebe upoznao
+al' to tada nisam shvatio
+Ne gledaj me da ne poludim
+jos bi mog'o sve da pokvarim
+sad si ista kao i ja, idu godine
+budi s drugim, budi bez mene
+Ref.</t>
+  </si>
+  <si>
+    <t>Refužo</t>
+  </si>
+  <si>
+    <t>Dalmatino</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>[Strofa 1]
+Blago mome oku šta te gleda
+Ti mi stižeš k'o najljepša vijest
+Šta nebesa nisu kocka leda
+Za naš stol ćeš skupa sa mnom sjest
+Blagoslivljan korak di si prošla
+Svaku stopu, treptaj oka tvog
+Fala nebu šta si meni došla
+A priko praga te prinija sam Bog
+[Refren]
+Moje sunce, moja bila ružo
+Oni šta se vole znaju to
+Samo jubav izuva postole
+I ka' rukon skida svaku bol
+Moje sunce, moja bila ružo
+Oni šta se vole znaju to
+Da se jubav ne daje refužo
+I na fete ne stavlja na stol
+[Strofa 2]
+I kad sunce potone u more
+Ja mu ne dan da dotakne dno
+Jer bi more, podivljalo i bisno
+Srcu mome bilo pretisno
+You might also like
+Bozic Bijeli
+Dalmatino
+Bad Bunny - DtMF (English Translation)
+Genius English Translations
+Risk It All
+Bruno Mars
+[Refren]
+Moje sunce, moja bila ružo
+Oni šta sе vole znaju to
+Samo jubav izuva postole
+I ka' rukon skida svaku bol
+Moje suncе, moja bila ružo
+Oni šta se vole znaju to
+Samo jubav izuva postole
+I ka rukon skida svaku bol
+[Refren]
+Moje sunce, moja bila ružo
+Oni šta se vole znaju to
+Samo jubav izuva postole
+I ka' rukon skida svaku bol
+(Moje sunce)
+Moja bila ružo
+Oni šta se vole znaju to
+Da se jubav ne daje refužo
+I na fete ne stavlja na stol
+[Završetak]
+Da se jubav ne daje refužo
+I na fete ne stavlja na stol</t>
   </si>
 </sst>
 </file>
@@ -901,280 +1043,399 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:O102"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="6" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.1640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="255.83203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.6640625" customWidth="1"/>
+    <col min="9" max="9" width="46.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="13.1640625" customWidth="1"/>
+    <col min="14" max="14" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:15" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
+      <c r="F2" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+    </row>
+    <row r="3" spans="1:15" ht="320" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+    </row>
+    <row r="4" spans="1:15" s="4" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A4" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="320" x14ac:dyDescent="0.2">
-      <c r="A3" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" s="4" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A4" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>10</v>
-      </c>
       <c r="E4" s="5" t="s">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>18</v>
       </c>
+      <c r="G4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>50</v>
+      </c>
       <c r="I4" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="J4" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" s="4" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A5" s="5" t="s">
         <v>19</v>
       </c>
+      <c r="B5" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>35</v>
+      </c>
     </row>
-    <row r="5" spans="1:12" s="4" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A5" s="5" t="s">
+    <row r="6" spans="1:15" s="4" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A6" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="H6" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" s="4" customFormat="1" ht="350" x14ac:dyDescent="0.2">
+      <c r="A7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" s="5" t="s">
+      <c r="C7" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F5" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>19</v>
+      <c r="D7" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:12" s="4" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A6" s="5" t="s">
+    <row r="8" spans="1:15" s="4" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A8" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C6" s="5" t="s">
+      <c r="C8" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" s="4" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A9" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="5" t="s">
+      <c r="B9" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F6" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>19</v>
+      <c r="D9" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:12" s="4" customFormat="1" ht="350" x14ac:dyDescent="0.2">
-      <c r="A7" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>19</v>
+    <row r="10" spans="1:15" s="4" customFormat="1" ht="365" x14ac:dyDescent="0.2">
+      <c r="A10" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:12" s="4" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A8" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="J8" s="5" t="s">
-        <v>19</v>
+    <row r="11" spans="1:15" s="4" customFormat="1" ht="365" x14ac:dyDescent="0.2">
+      <c r="A11" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:12" s="4" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A9" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D9" s="5" t="s">
+    <row r="12" spans="1:15" s="4" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A12" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G12" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="J9" s="5" t="s">
-        <v>19</v>
+      <c r="H12" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>67</v>
       </c>
     </row>
-    <row r="10" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="11" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="12" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="13" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="14" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="15" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="16" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="13" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="14" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="15" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="16" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="17" s="4" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="18" s="4" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="19" s="4" customFormat="1" x14ac:dyDescent="0.2"/>

</xml_diff>